<commit_message>
feat: integrate device fingerprinting, admin inline editing, stats recalculation, fix admin font encoding, and update docs
</commit_message>
<xml_diff>
--- a/legacy/PICKLEBALL RANKING.xlsx
+++ b/legacy/PICKLEBALL RANKING.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="124">
   <si>
     <t>player_id</t>
   </si>
@@ -63,6 +63,12 @@
     <t>Nguyễn Ngọc Văn</t>
   </si>
   <si>
+    <t>__GUEST__</t>
+  </si>
+  <si>
+    <t>khách</t>
+  </si>
+  <si>
     <t>match_id</t>
   </si>
   <si>
@@ -153,6 +159,48 @@
     <t>M1777894855821</t>
   </si>
   <si>
+    <t>M1777978420578</t>
+  </si>
+  <si>
+    <t>M1777978752045</t>
+  </si>
+  <si>
+    <t>M1777979508388</t>
+  </si>
+  <si>
+    <t>M1777980114060</t>
+  </si>
+  <si>
+    <t>M1777980791926</t>
+  </si>
+  <si>
+    <t>M1778063354486</t>
+  </si>
+  <si>
+    <t>M1778065754883</t>
+  </si>
+  <si>
+    <t>M1778065845619</t>
+  </si>
+  <si>
+    <t>M1778068171302</t>
+  </si>
+  <si>
+    <t>M1778075138730</t>
+  </si>
+  <si>
+    <t>M1778075296691</t>
+  </si>
+  <si>
+    <t>M1778075627431</t>
+  </si>
+  <si>
+    <t>M1778075656261</t>
+  </si>
+  <si>
+    <t>M1778077637563</t>
+  </si>
+  <si>
     <t>key</t>
   </si>
   <si>
@@ -180,7 +228,7 @@
     <t>last_action</t>
   </si>
   <si>
-    <t>add_match</t>
+    <t>delete_player</t>
   </si>
   <si>
     <t>global_version</t>
@@ -715,6 +763,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -732,36 +791,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3">
         <v>46140.72798674769</v>
@@ -785,12 +844,12 @@
         <v>8.0</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3">
         <v>46140.73421962963</v>
@@ -814,12 +873,12 @@
         <v>6.0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" s="3">
         <v>46140.73700702546</v>
@@ -843,12 +902,12 @@
         <v>1.0</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3">
         <v>46140.743899340276</v>
@@ -872,12 +931,12 @@
         <v>4.0</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3">
         <v>46140.76307925926</v>
@@ -901,12 +960,12 @@
         <v>5.0</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3">
         <v>46140.76388290509</v>
@@ -930,12 +989,12 @@
         <v>10.0</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="3">
         <v>46140.76525894676</v>
@@ -959,12 +1018,12 @@
         <v>4.0</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B9" s="3">
         <v>46140.77092585649</v>
@@ -988,12 +1047,12 @@
         <v>4.0</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B10" s="3">
         <v>46141.72873754629</v>
@@ -1017,12 +1076,12 @@
         <v>5.0</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B11" s="3">
         <v>46141.73779349537</v>
@@ -1046,12 +1105,12 @@
         <v>9.0</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B12" s="3">
         <v>46141.74176315972</v>
@@ -1075,12 +1134,12 @@
         <v>0.0</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13" s="3">
         <v>46141.750260810186</v>
@@ -1104,12 +1163,12 @@
         <v>7.0</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B14" s="3">
         <v>46141.759347847226</v>
@@ -1133,12 +1192,12 @@
         <v>2.0</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B15" s="3">
         <v>46146.72649137731</v>
@@ -1162,12 +1221,12 @@
         <v>5.0</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B16" s="3">
         <v>46146.734277627314</v>
@@ -1191,12 +1250,12 @@
         <v>3.0</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B17" s="3">
         <v>46146.74718006945</v>
@@ -1220,12 +1279,12 @@
         <v>12.0</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B18" s="3">
         <v>46146.756049930555</v>
@@ -1249,12 +1308,12 @@
         <v>7.0</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B19" s="3">
         <v>46146.764099293985</v>
@@ -1278,12 +1337,12 @@
         <v>8.0</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B20" s="3">
         <v>46146.769729733795</v>
@@ -1307,12 +1366,12 @@
         <v>2.0</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="3">
         <v>46146.778423854164</v>
@@ -1336,7 +1395,413 @@
         <v>10.0</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46147.74560854166</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46147.74944496527</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G23" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46147.75819893519</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46147.76520902778</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H25" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46147.77305469908</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H26" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46148.728639884255</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G27" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="H27" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46148.75642225695</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G28" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="H28" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46148.75747244213</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H29" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46148.78439006944</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H30" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46148.86503159722</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H31" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46148.86685984954</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H32" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46148.8706878588</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G33" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H33" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="3">
+        <v>46148.87102153935</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H34" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46148.89395327546</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H35" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1353,23 +1818,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1">
         <v>5000.0</v>
@@ -1393,39 +1858,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="B5" s="1">
         <v>1.777043938961E12</v>
@@ -1449,47 +1914,47 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1">
-        <v>1.777894855945E12</v>
+        <v>1.778078127584E12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B4" s="1">
-        <v>1.777894855945E12</v>
+        <v>1.778078127584E12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="B5" s="1">
-        <v>1.777894855945E12</v>
+        <v>1.778078127584E12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B6" s="1">
         <v>1.77739598107E12</v>
@@ -1497,15 +1962,15 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="B7" s="1">
-        <v>1.777395981747E12</v>
+        <v>1.778078127584E12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="B8" s="1">
         <v>1.777395983376E12</v>
@@ -1513,7 +1978,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="B9" s="1">
         <v>1.777400004237E12</v>
@@ -1521,7 +1986,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="B10" s="1">
         <v>1.777395985073E12</v>
@@ -1529,7 +1994,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B11" s="1">
         <v>1.777395986213E12</v>
@@ -1537,7 +2002,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="B12" s="1">
         <v>1.77739598691E12</v>
@@ -1545,15 +2010,15 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="B13" s="1">
-        <v>1.777894273916E12</v>
+        <v>1.778078127584E12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="B14" s="1">
         <v>1.777395989835E12</v>
@@ -1573,48 +2038,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="B2" s="3">
         <v>46137.02012170139</v>
@@ -1638,16 +2103,16 @@
         <v>0.0</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J2" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M2" s="1" t="b">
         <v>1</v>
@@ -1655,7 +2120,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3">
         <v>46137.02004299768</v>
@@ -1679,16 +2144,16 @@
         <v>0.0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J3" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M3" s="1" t="b">
         <v>1</v>
@@ -1696,7 +2161,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="B4" s="3">
         <v>46137.02003662037</v>
@@ -1720,16 +2185,16 @@
         <v>0.0</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J4" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M4" s="1" t="b">
         <v>1</v>
@@ -1737,7 +2202,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="B5" s="3">
         <v>46137.01998991898</v>
@@ -1761,16 +2226,16 @@
         <v>0.0</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J5" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M5" s="1" t="b">
         <v>1</v>
@@ -1778,7 +2243,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B6" s="3">
         <v>46137.07473655093</v>
@@ -1802,16 +2267,16 @@
         <v>0.0</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J6" s="3">
         <v>46137.07509039352</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M6" s="1" t="b">
         <v>0</v>
@@ -1819,7 +2284,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="B7" s="3">
         <v>46137.068427060185</v>
@@ -1843,16 +2308,16 @@
         <v>0.0</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J7" s="3">
         <v>46137.07509039352</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M7" s="1" t="b">
         <v>0</v>
@@ -1860,7 +2325,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="B8" s="3">
         <v>46137.78489793981</v>
@@ -1884,16 +2349,16 @@
         <v>0.0</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J8" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M8" s="1" t="b">
         <v>0</v>
@@ -1901,7 +2366,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>46137.60813393518</v>
@@ -1925,16 +2390,16 @@
         <v>0.0</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J9" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M9" s="1" t="b">
         <v>0</v>
@@ -1942,7 +2407,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="B10" s="3">
         <v>46137.607969895835</v>
@@ -1966,16 +2431,16 @@
         <v>0.0</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J10" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M10" s="1" t="b">
         <v>0</v>
@@ -1983,7 +2448,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="B11" s="3">
         <v>46137.60751290509</v>
@@ -2007,16 +2472,16 @@
         <v>0.0</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J11" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M11" s="1" t="b">
         <v>0</v>
@@ -2024,7 +2489,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="B12" s="3">
         <v>46137.60680480324</v>
@@ -2048,16 +2513,16 @@
         <v>0.0</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J12" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M12" s="1" t="b">
         <v>0</v>
@@ -2065,7 +2530,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B13" s="3">
         <v>46137.60123398148</v>
@@ -2089,16 +2554,16 @@
         <v>0.0</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J13" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M13" s="1" t="b">
         <v>0</v>
@@ -2106,7 +2571,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B14" s="3">
         <v>46137.601130740746</v>
@@ -2130,16 +2595,16 @@
         <v>0.0</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J14" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M14" s="1" t="b">
         <v>0</v>
@@ -2147,7 +2612,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="B15" s="3">
         <v>46137.400231458334</v>
@@ -2171,16 +2636,16 @@
         <v>0.0</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J15" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M15" s="1" t="b">
         <v>0</v>
@@ -2188,7 +2653,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="B16" s="3">
         <v>46137.40018256944</v>
@@ -2212,16 +2677,16 @@
         <v>0.0</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J16" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M16" s="1" t="b">
         <v>0</v>
@@ -2229,7 +2694,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="B17" s="3">
         <v>46137.40017483797</v>
@@ -2253,16 +2718,16 @@
         <v>0.0</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J17" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M17" s="1" t="b">
         <v>0</v>
@@ -2270,7 +2735,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="B18" s="3">
         <v>46137.40016186342</v>
@@ -2294,16 +2759,16 @@
         <v>0.0</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J18" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M18" s="1" t="b">
         <v>0</v>
@@ -2311,16 +2776,16 @@
     </row>
     <row r="19">
       <c r="I19" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J19" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M19" s="1" t="b">
         <v>0</v>
@@ -2328,7 +2793,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="B20" s="3">
         <v>46137.40011466436</v>
@@ -2352,16 +2817,16 @@
         <v>0.0</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="J20" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M20" s="1" t="b">
         <v>0</v>
@@ -2369,7 +2834,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B21" s="3">
         <v>46137.39544247685</v>
@@ -2393,16 +2858,16 @@
         <v>0.0</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J21" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M21" s="1" t="b">
         <v>0</v>
@@ -2410,7 +2875,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="B22" s="3">
         <v>46137.38264790509</v>
@@ -2434,16 +2899,16 @@
         <v>0.0</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J22" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M22" s="1" t="b">
         <v>0</v>
@@ -2451,7 +2916,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="B23" s="3">
         <v>46137.07635552083</v>
@@ -2475,16 +2940,16 @@
         <v>0.0</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J23" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M23" s="1" t="b">
         <v>0</v>
@@ -2492,7 +2957,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="B24" s="3">
         <v>46137.07632814815</v>
@@ -2516,16 +2981,16 @@
         <v>0.0</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J24" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M24" s="1" t="b">
         <v>0</v>
@@ -2533,7 +2998,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="B25" s="3">
         <v>46137.07629898148</v>
@@ -2557,16 +3022,16 @@
         <v>0.0</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J25" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M25" s="1" t="b">
         <v>0</v>
@@ -2574,7 +3039,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="B26" s="3">
         <v>46137.07625113426</v>
@@ -2598,16 +3063,16 @@
         <v>0.0</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J26" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M26" s="1" t="b">
         <v>0</v>
@@ -2615,7 +3080,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="B27" s="3">
         <v>46137.07622623842</v>
@@ -2639,16 +3104,16 @@
         <v>0.0</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J27" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M27" s="1" t="b">
         <v>0</v>
@@ -2656,7 +3121,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B28" s="3">
         <v>46137.076213946755</v>
@@ -2680,16 +3145,16 @@
         <v>0.0</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J28" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M28" s="1" t="b">
         <v>0</v>
@@ -2697,7 +3162,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B29" s="3">
         <v>46137.076150775465</v>
@@ -2721,16 +3186,16 @@
         <v>0.0</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J29" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M29" s="1" t="b">
         <v>0</v>
@@ -2738,7 +3203,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="B30" s="3">
         <v>46137.07609715278</v>
@@ -2762,16 +3227,16 @@
         <v>0.0</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J30" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M30" s="1" t="b">
         <v>0</v>
@@ -2779,7 +3244,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B31" s="3">
         <v>46137.076082141204</v>
@@ -2803,16 +3268,16 @@
         <v>0.0</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J31" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M31" s="1" t="b">
         <v>0</v>
@@ -2820,7 +3285,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="B32" s="3">
         <v>46137.07601829861</v>
@@ -2844,16 +3309,16 @@
         <v>0.0</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J32" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M32" s="1" t="b">
         <v>0</v>
@@ -2861,7 +3326,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="B33" s="3">
         <v>46137.07600688658</v>
@@ -2885,16 +3350,16 @@
         <v>0.0</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J33" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M33" s="1" t="b">
         <v>0</v>
@@ -2902,7 +3367,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="B34" s="3">
         <v>46137.07593449074</v>
@@ -2926,16 +3391,16 @@
         <v>0.0</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J34" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M34" s="1" t="b">
         <v>0</v>
@@ -2943,7 +3408,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="B35" s="3">
         <v>46137.07593170139</v>
@@ -2967,16 +3432,16 @@
         <v>0.0</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J35" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M35" s="1" t="b">
         <v>0</v>
@@ -2984,7 +3449,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="B36" s="3">
         <v>46137.07589289352</v>
@@ -3008,16 +3473,16 @@
         <v>0.0</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J36" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M36" s="1" t="b">
         <v>0</v>
@@ -3025,7 +3490,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="B37" s="3">
         <v>46137.07581966435</v>
@@ -3049,16 +3514,16 @@
         <v>0.0</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J37" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="M37" s="1" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
feat: revamp leaderboard insight labels and expand variation lists
</commit_message>
<xml_diff>
--- a/legacy/PICKLEBALL RANKING.xlsx
+++ b/legacy/PICKLEBALL RANKING.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="141">
   <si>
     <t>player_id</t>
   </si>
@@ -69,6 +69,12 @@
     <t>khách</t>
   </si>
   <si>
+    <t>P007</t>
+  </si>
+  <si>
+    <t>Trần Ngọc Hà</t>
+  </si>
+  <si>
     <t>match_id</t>
   </si>
   <si>
@@ -201,6 +207,51 @@
     <t>M1778077637563</t>
   </si>
   <si>
+    <t>M1778161581585</t>
+  </si>
+  <si>
+    <t>M1778161617980</t>
+  </si>
+  <si>
+    <t>M1778161648730</t>
+  </si>
+  <si>
+    <t>M1778161675850</t>
+  </si>
+  <si>
+    <t>M1778161692693</t>
+  </si>
+  <si>
+    <t>M1778323910745</t>
+  </si>
+  <si>
+    <t>M1778323934615</t>
+  </si>
+  <si>
+    <t>M1778323959564</t>
+  </si>
+  <si>
+    <t>M1778324226863</t>
+  </si>
+  <si>
+    <t>M1778324805427</t>
+  </si>
+  <si>
+    <t>M1778326531895</t>
+  </si>
+  <si>
+    <t>M1778326546835</t>
+  </si>
+  <si>
+    <t>M1778326921047</t>
+  </si>
+  <si>
+    <t>M1778329206331</t>
+  </si>
+  <si>
+    <t>M1778330461393</t>
+  </si>
+  <si>
     <t>key</t>
   </si>
   <si>
@@ -228,7 +279,7 @@
     <t>last_action</t>
   </si>
   <si>
-    <t>delete_player</t>
+    <t>add_match</t>
   </si>
   <si>
     <t>global_version</t>
@@ -774,6 +825,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -791,36 +853,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B2" s="3">
         <v>46140.72798674769</v>
@@ -844,12 +906,12 @@
         <v>8.0</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3">
         <v>46140.73421962963</v>
@@ -873,12 +935,12 @@
         <v>6.0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B4" s="3">
         <v>46140.73700702546</v>
@@ -902,12 +964,12 @@
         <v>1.0</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" s="3">
         <v>46140.743899340276</v>
@@ -931,12 +993,12 @@
         <v>4.0</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="3">
         <v>46140.76307925926</v>
@@ -960,12 +1022,12 @@
         <v>5.0</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" s="3">
         <v>46140.76388290509</v>
@@ -989,12 +1051,12 @@
         <v>10.0</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8" s="3">
         <v>46140.76525894676</v>
@@ -1018,12 +1080,12 @@
         <v>4.0</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3">
         <v>46140.77092585649</v>
@@ -1047,12 +1109,12 @@
         <v>4.0</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B10" s="3">
         <v>46141.72873754629</v>
@@ -1076,12 +1138,12 @@
         <v>5.0</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B11" s="3">
         <v>46141.73779349537</v>
@@ -1105,12 +1167,12 @@
         <v>9.0</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" s="3">
         <v>46141.74176315972</v>
@@ -1134,12 +1196,12 @@
         <v>0.0</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B13" s="3">
         <v>46141.750260810186</v>
@@ -1163,12 +1225,12 @@
         <v>7.0</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" s="3">
         <v>46141.759347847226</v>
@@ -1192,12 +1254,12 @@
         <v>2.0</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B15" s="3">
         <v>46146.72649137731</v>
@@ -1221,12 +1283,12 @@
         <v>5.0</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B16" s="3">
         <v>46146.734277627314</v>
@@ -1250,12 +1312,12 @@
         <v>3.0</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B17" s="3">
         <v>46146.74718006945</v>
@@ -1279,12 +1341,12 @@
         <v>12.0</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B18" s="3">
         <v>46146.756049930555</v>
@@ -1308,12 +1370,12 @@
         <v>7.0</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B19" s="3">
         <v>46146.764099293985</v>
@@ -1337,12 +1399,12 @@
         <v>8.0</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B20" s="3">
         <v>46146.769729733795</v>
@@ -1366,12 +1428,12 @@
         <v>2.0</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" s="3">
         <v>46146.778423854164</v>
@@ -1395,12 +1457,12 @@
         <v>10.0</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B22" s="3">
         <v>46147.74560854166</v>
@@ -1424,12 +1486,12 @@
         <v>1.0</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B23" s="3">
         <v>46147.74944496527</v>
@@ -1453,12 +1515,12 @@
         <v>9.0</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B24" s="3">
         <v>46147.75819893519</v>
@@ -1482,12 +1544,12 @@
         <v>8.0</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B25" s="3">
         <v>46147.76520902778</v>
@@ -1511,12 +1573,12 @@
         <v>7.0</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" s="3">
         <v>46147.77305469908</v>
@@ -1540,12 +1602,12 @@
         <v>5.0</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B27" s="3">
         <v>46148.728639884255</v>
@@ -1557,7 +1619,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>3</v>
@@ -1569,12 +1631,12 @@
         <v>9.0</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B28" s="3">
         <v>46148.75642225695</v>
@@ -1586,7 +1648,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>3</v>
@@ -1598,12 +1660,12 @@
         <v>10.0</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B29" s="3">
         <v>46148.75747244213</v>
@@ -1627,12 +1689,12 @@
         <v>4.0</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B30" s="3">
         <v>46148.78439006944</v>
@@ -1656,12 +1718,12 @@
         <v>5.0</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B31" s="3">
         <v>46148.86503159722</v>
@@ -1676,7 +1738,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G31" s="4">
         <v>11.0</v>
@@ -1685,12 +1747,12 @@
         <v>2.0</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B32" s="3">
         <v>46148.86685984954</v>
@@ -1714,12 +1776,12 @@
         <v>4.0</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B33" s="3">
         <v>46148.8706878588</v>
@@ -1734,7 +1796,7 @@
         <v>5</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G33" s="4">
         <v>11.0</v>
@@ -1743,12 +1805,12 @@
         <v>5.0</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B34" s="3">
         <v>46148.87102153935</v>
@@ -1763,7 +1825,7 @@
         <v>5</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G34" s="4">
         <v>11.0</v>
@@ -1772,12 +1834,12 @@
         <v>8.0</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B35" s="3">
         <v>46148.89395327546</v>
@@ -1792,7 +1854,7 @@
         <v>3</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G35" s="4">
         <v>11.0</v>
@@ -1801,7 +1863,442 @@
         <v>3.0</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46149.86552760417</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H36" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="3">
+        <v>46149.86594884259</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H37" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46149.866304745374</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G38" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H38" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46149.86661863426</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G39" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="H39" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40" s="3">
+        <v>46149.86681357639</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H40" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="3">
+        <v>46151.744337337965</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G41" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H41" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B42" s="3">
+        <v>46151.74461359954</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H42" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B43" s="3">
+        <v>46151.74490236111</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G43" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H43" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B44" s="3">
+        <v>46151.74799609954</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H44" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="3">
+        <v>46151.75469244213</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G45" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H45" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B46" s="3">
+        <v>46151.77467471064</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G46" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H46" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B47" s="3">
+        <v>46151.77484762731</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G47" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H47" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B48" s="3">
+        <v>46151.77917878472</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G48" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="H48" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49" s="3">
+        <v>46151.80562883102</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H49" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50" s="3">
+        <v>46151.82015501158</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="H50" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1818,23 +2315,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="B3" s="1">
         <v>5000.0</v>
@@ -1858,39 +2355,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B5" s="1">
         <v>1.777043938961E12</v>
@@ -1914,47 +2411,47 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="B2" s="1">
-        <v>1.778078127584E12</v>
+        <v>1.778330461467E12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="B4" s="1">
-        <v>1.778078127584E12</v>
+        <v>1.778330461467E12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="B5" s="1">
-        <v>1.778078127584E12</v>
+        <v>1.778330461467E12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="B6" s="1">
         <v>1.77739598107E12</v>
@@ -1962,15 +2459,15 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="B7" s="1">
-        <v>1.778078127584E12</v>
+        <v>1.778144122213E12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="B8" s="1">
         <v>1.777395983376E12</v>
@@ -1978,7 +2475,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="B9" s="1">
         <v>1.777400004237E12</v>
@@ -1986,7 +2483,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="B10" s="1">
         <v>1.777395985073E12</v>
@@ -1994,7 +2491,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="B11" s="1">
         <v>1.777395986213E12</v>
@@ -2002,7 +2499,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B12" s="1">
         <v>1.77739598691E12</v>
@@ -2010,7 +2507,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B13" s="1">
         <v>1.778078127584E12</v>
@@ -2018,7 +2515,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="B14" s="1">
         <v>1.777395989835E12</v>
@@ -2038,48 +2535,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="B2" s="3">
         <v>46137.02012170139</v>
@@ -2103,16 +2600,16 @@
         <v>0.0</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J2" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M2" s="1" t="b">
         <v>1</v>
@@ -2120,7 +2617,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="B3" s="3">
         <v>46137.02004299768</v>
@@ -2144,16 +2641,16 @@
         <v>0.0</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J3" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M3" s="1" t="b">
         <v>1</v>
@@ -2161,7 +2658,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B4" s="3">
         <v>46137.02003662037</v>
@@ -2185,16 +2682,16 @@
         <v>0.0</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J4" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M4" s="1" t="b">
         <v>1</v>
@@ -2202,7 +2699,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="B5" s="3">
         <v>46137.01998991898</v>
@@ -2226,16 +2723,16 @@
         <v>0.0</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J5" s="3">
         <v>46137.02040016204</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M5" s="1" t="b">
         <v>1</v>
@@ -2243,7 +2740,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B6" s="3">
         <v>46137.07473655093</v>
@@ -2267,16 +2764,16 @@
         <v>0.0</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J6" s="3">
         <v>46137.07509039352</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M6" s="1" t="b">
         <v>0</v>
@@ -2284,7 +2781,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="B7" s="3">
         <v>46137.068427060185</v>
@@ -2308,16 +2805,16 @@
         <v>0.0</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J7" s="3">
         <v>46137.07509039352</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M7" s="1" t="b">
         <v>0</v>
@@ -2325,7 +2822,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B8" s="3">
         <v>46137.78489793981</v>
@@ -2349,16 +2846,16 @@
         <v>0.0</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J8" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M8" s="1" t="b">
         <v>0</v>
@@ -2366,7 +2863,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B9" s="3">
         <v>46137.60813393518</v>
@@ -2390,16 +2887,16 @@
         <v>0.0</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J9" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M9" s="1" t="b">
         <v>0</v>
@@ -2407,7 +2904,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B10" s="3">
         <v>46137.607969895835</v>
@@ -2431,16 +2928,16 @@
         <v>0.0</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J10" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M10" s="1" t="b">
         <v>0</v>
@@ -2448,7 +2945,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="B11" s="3">
         <v>46137.60751290509</v>
@@ -2472,16 +2969,16 @@
         <v>0.0</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J11" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M11" s="1" t="b">
         <v>0</v>
@@ -2489,7 +2986,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="B12" s="3">
         <v>46137.60680480324</v>
@@ -2513,16 +3010,16 @@
         <v>0.0</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J12" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M12" s="1" t="b">
         <v>0</v>
@@ -2530,7 +3027,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B13" s="3">
         <v>46137.60123398148</v>
@@ -2554,16 +3051,16 @@
         <v>0.0</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J13" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M13" s="1" t="b">
         <v>0</v>
@@ -2571,7 +3068,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B14" s="3">
         <v>46137.601130740746</v>
@@ -2595,16 +3092,16 @@
         <v>0.0</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J14" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M14" s="1" t="b">
         <v>0</v>
@@ -2612,7 +3109,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="B15" s="3">
         <v>46137.400231458334</v>
@@ -2636,16 +3133,16 @@
         <v>0.0</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J15" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M15" s="1" t="b">
         <v>0</v>
@@ -2653,7 +3150,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="B16" s="3">
         <v>46137.40018256944</v>
@@ -2677,16 +3174,16 @@
         <v>0.0</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J16" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M16" s="1" t="b">
         <v>0</v>
@@ -2694,7 +3191,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="B17" s="3">
         <v>46137.40017483797</v>
@@ -2718,16 +3215,16 @@
         <v>0.0</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J17" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M17" s="1" t="b">
         <v>0</v>
@@ -2735,7 +3232,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B18" s="3">
         <v>46137.40016186342</v>
@@ -2759,16 +3256,16 @@
         <v>0.0</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J18" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M18" s="1" t="b">
         <v>0</v>
@@ -2776,16 +3273,16 @@
     </row>
     <row r="19">
       <c r="I19" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J19" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M19" s="1" t="b">
         <v>0</v>
@@ -2793,7 +3290,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B20" s="3">
         <v>46137.40011466436</v>
@@ -2817,16 +3314,16 @@
         <v>0.0</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="J20" s="3">
         <v>46140.45943503472</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M20" s="1" t="b">
         <v>0</v>
@@ -2834,7 +3331,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B21" s="3">
         <v>46137.39544247685</v>
@@ -2858,16 +3355,16 @@
         <v>0.0</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J21" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M21" s="1" t="b">
         <v>0</v>
@@ -2875,7 +3372,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B22" s="3">
         <v>46137.38264790509</v>
@@ -2899,16 +3396,16 @@
         <v>0.0</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J22" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M22" s="1" t="b">
         <v>0</v>
@@ -2916,7 +3413,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="B23" s="3">
         <v>46137.07635552083</v>
@@ -2940,16 +3437,16 @@
         <v>0.0</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J23" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M23" s="1" t="b">
         <v>0</v>
@@ -2957,7 +3454,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B24" s="3">
         <v>46137.07632814815</v>
@@ -2981,16 +3478,16 @@
         <v>0.0</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J24" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M24" s="1" t="b">
         <v>0</v>
@@ -2998,7 +3495,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B25" s="3">
         <v>46137.07629898148</v>
@@ -3022,16 +3519,16 @@
         <v>0.0</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J25" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M25" s="1" t="b">
         <v>0</v>
@@ -3039,7 +3536,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="B26" s="3">
         <v>46137.07625113426</v>
@@ -3063,16 +3560,16 @@
         <v>0.0</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J26" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M26" s="1" t="b">
         <v>0</v>
@@ -3080,7 +3577,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="B27" s="3">
         <v>46137.07622623842</v>
@@ -3104,16 +3601,16 @@
         <v>0.0</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J27" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M27" s="1" t="b">
         <v>0</v>
@@ -3121,7 +3618,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="B28" s="3">
         <v>46137.076213946755</v>
@@ -3145,16 +3642,16 @@
         <v>0.0</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J28" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M28" s="1" t="b">
         <v>0</v>
@@ -3162,7 +3659,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="B29" s="3">
         <v>46137.076150775465</v>
@@ -3186,16 +3683,16 @@
         <v>0.0</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J29" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M29" s="1" t="b">
         <v>0</v>
@@ -3203,7 +3700,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="B30" s="3">
         <v>46137.07609715278</v>
@@ -3227,16 +3724,16 @@
         <v>0.0</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J30" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M30" s="1" t="b">
         <v>0</v>
@@ -3244,7 +3741,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="B31" s="3">
         <v>46137.076082141204</v>
@@ -3268,16 +3765,16 @@
         <v>0.0</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J31" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M31" s="1" t="b">
         <v>0</v>
@@ -3285,7 +3782,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="B32" s="3">
         <v>46137.07601829861</v>
@@ -3309,16 +3806,16 @@
         <v>0.0</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J32" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M32" s="1" t="b">
         <v>0</v>
@@ -3326,7 +3823,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="B33" s="3">
         <v>46137.07600688658</v>
@@ -3350,16 +3847,16 @@
         <v>0.0</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J33" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M33" s="1" t="b">
         <v>0</v>
@@ -3367,7 +3864,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3">
         <v>46137.07593449074</v>
@@ -3391,16 +3888,16 @@
         <v>0.0</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J34" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M34" s="1" t="b">
         <v>0</v>
@@ -3408,7 +3905,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="B35" s="3">
         <v>46137.07593170139</v>
@@ -3432,16 +3929,16 @@
         <v>0.0</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J35" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M35" s="1" t="b">
         <v>0</v>
@@ -3449,7 +3946,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="B36" s="3">
         <v>46137.07589289352</v>
@@ -3473,16 +3970,16 @@
         <v>0.0</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J36" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M36" s="1" t="b">
         <v>0</v>
@@ -3490,7 +3987,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="B37" s="3">
         <v>46137.07581966435</v>
@@ -3514,16 +4011,16 @@
         <v>0.0</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J37" s="3">
         <v>46140.45947862268</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="M37" s="1" t="b">
         <v>0</v>

</xml_diff>